<commit_message>
Document the new test workflows and the source-sheet findings
Three no-cost workflows were added over this session and were not listed. The
un_sites notes now record what was verified on 11 August: which agency sites
refuse automated requests, and that a feed_url beats scraping a listing page.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sources/sources.xlsx
+++ b/sources/sources.xlsx
@@ -2622,7 +2622,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F15" s="5" t="n"/>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>listing page yields no links to our parser; ReliefWeb's API needs an approved appname (checked 11 Aug 2026)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Fill the roster from the UN Mongolia team pages
The roster sheet has been empty since the project started, and every run said
so: an article quoting the Resident Coordinator by name, without also writing
'United Nations', was invisible to the collector. Eleven names are now in,
taken from mongolia.un.org's team and RCO pages on 11 August 2026, with the
Cyrillic forms from the same pages' Mongolian versions — the aliases are the
load-bearing part, since local coverage rarely uses Latin script.

Where the press spells a name differently from our own site, both are listed:
the UNDP Resident Representative appears as Лионель Лоуренс in Mongolian
coverage (mnb.mn, 5 August 2026) and as Лионел Лорон on mongolia.un.org.

These are current officeholders, not a permanent list — the notes column
records when each was checked so the office can tell when it went stale.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sources/sources.xlsx
+++ b/sources/sources.xlsx
@@ -1926,12 +1926,12 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>EXAMPLE — delete this row</t>
+          <t>Jaap van Hierden</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Resident Coordinator</t>
+          <t>UN Resident Coordinator</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Ж. Смит, Smith Jane, J. Smith</t>
+          <t>Яап ван Хиердэн, ван Хиердэн, Jaap Van Hierden</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -1951,27 +1951,31 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>How a row should look</t>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages; RC since 1 Jan 2025</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>&lt;FILL IN&gt;</t>
+          <t>Beate Dastel</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>UN Resident Coordinator</t>
+          <t>UNICEF Representative</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>UNRCO</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n"/>
+          <t>UNICEF</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Беате Дастел, Дастел</t>
+        </is>
+      </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1979,225 +1983,297 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Add the real name and every Cyrillic spelling</t>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages; took office Feb 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>&lt;FILL IN&gt;</t>
+          <t>Lionel Laurens</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Head of Office</t>
+          <t>UNDP Resident Representative</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>UNICEF</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n"/>
+          <t>UNDP</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Лионель Лоуренс, Лионел Лорон, Лоуренс</t>
+        </is>
+      </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages; press spelling from mnb.mn 5 Aug 2026 differs from the UN site</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>&lt;FILL IN&gt;</t>
+          <t>Socorro Escalante</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Head of Office</t>
+          <t>WHO Representative</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>UNDP</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n"/>
+          <t>WHO</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Сокорро Эскалантэ, Эскалантэ</t>
+        </is>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>&lt;FILL IN&gt;</t>
+          <t>Yoko Fujimura</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Head of Office</t>
+          <t>IOM Chief of Mission</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>UNFPA</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="n"/>
+          <t>IOM</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Ёко Фүжимүра, Фүжимүра</t>
+        </is>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>&lt;FILL IN&gt;</t>
+          <t>Qingyun Diao</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Representative</t>
+          <t>FAO Representative</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>WHO</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n"/>
+          <t>FAO</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Чинюнь Дяо, Дяо</t>
+        </is>
+      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>&lt;FILL IN&gt;</t>
+          <t>Khalid Sharifi</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Head of Office</t>
+          <t>UNFPA Head of Office</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>IOM</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n"/>
+          <t>UNFPA</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Халид Шарифи, Шарифи</t>
+        </is>
+      </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F9" s="5" t="n"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>&lt;FILL IN&gt;</t>
+          <t>Ganbold Baasanjav</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Representative</t>
+          <t>Head, ESCAP East and North-East Asia Office</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>FAO</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="n"/>
+          <t>ESCAP</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Ганболд Баасанжав, Б.Ганболд</t>
+        </is>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F10" s="5" t="n"/>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>&lt;FILL IN&gt;</t>
+          <t>Doljinsuren Jambal</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Head of Office</t>
+          <t>Head of the Resident Coordinator's Office</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n"/>
+          <t>UNRCO</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Должинсүрэн Жамбал, Ж.Должинсүрэн</t>
+        </is>
+      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="n"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>&lt;FILL IN&gt;</t>
+          <t>Altangerel Choijoo</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Head of Office</t>
+          <t>National Human Rights Advisor</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>ILO</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n"/>
+          <t>UNRCO</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Алтангэрэл Чойжоо, Ч.Алтангэрэл</t>
+        </is>
+      </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>&lt;FILL IN&gt;</t>
+          <t>Soyolmaa Dolgor</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Head of Office</t>
+          <t>Development Coordination Officer, Communications</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>UN Women</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n"/>
+          <t>UNRCO</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Соёлмаа Долгор, Д.Соёлмаа</t>
+        </is>
+      </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>verified 11 Aug 2026 from mongolia.un.org team pages</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Require a full name before waiving the Mongolia check
Filling the roster surfaced a hole in the waiver added with it. A roster match
lets an article through without mentioning Mongolia, on the reasoning that a
profile of the Resident Coordinator need not repeat the country's name — but
the aliases included bare surnames, and "Шарифи" duly collected eleven
articles about unrelated Tajik and Iranian people as Mongolian media coverage.

Only a term of two or more words now earns the waiver, and the surname-only
aliases are out of the sheet. Mongolian initial+name forms (Ж.Должинсүрэн) are
kept and still count: the initial makes them specific.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sources/sources.xlsx
+++ b/sources/sources.xlsx
@@ -1973,7 +1973,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Беате Дастел, Дастел</t>
+          <t>Беате Дастел</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Лионель Лоуренс, Лионел Лорон, Лоуренс</t>
+          <t>Лионель Лоуренс, Лионел Лорон</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Сокорро Эскалантэ, Эскалантэ</t>
+          <t>Сокорро Эскалантэ</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Ёко Фүжимүра, Фүжимүра</t>
+          <t>Ёко Фүжимүра</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Чинюнь Дяо, Дяо</t>
+          <t>Чинюнь Дяо</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Халид Шарифи, Шарифи</t>
+          <t>Халид Шарифи</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">

</xml_diff>